<commit_message>
Add manual-research sheet to Excel export
Second sheet lists the 12 companies with no confident Apollo match, so
they're tracked alongside the verified contacts in one file rather than
only in chat.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA3eMoHLG5tHsDy3VcGJJG
</commit_message>
<xml_diff>
--- a/wealth_batch2_verified_contacts.xlsx
+++ b/wealth_batch2_verified_contacts.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Verified Contacts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Needs Manual Research" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verified Contacts'!$A$1:$E$39</definedName>
@@ -1502,4 +1503,178 @@
   <autoFilter ref="A1:E39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1st Commercial Credit</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Trilantic North America</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Presario Ventures</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cotton Creek Capital</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Quake Capital Partners</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>DynEvolve Capital</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Spindletop Capital</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Keyes Capital Group</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Mako Strategies</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Altamont Capital Partners</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Sunny River Management</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Swank Investments, Inc.</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild batch #2 results: web-research decision-makers, drop gatekeeper tier
Combines the credit-based enrichment with free web-research lookups
(company team/leadership pages, cross-validated against Apollo's
obfuscated records via resolve_candidate) to raise contact counts per
company - most companies now have 3-9 contacts instead of 1-2, without
spending additional Apollo credits beyond the original sample.

Output now excludes gatekeeper/EA-only rows per updated targeting -
decision-makers and marketing roles only. Excel export adds a Notes &
Caveats sheet flagging the handful of lower-confidence results (Peak Rock
Capital's secondary-domain contact, Capstone Capital Partners' ambiguous
match, CenterGate/8VC's inconsistent per-employee formats).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA3eMoHLG5tHsDy3VcGJJG
</commit_message>
<xml_diff>
--- a/wealth_batch2_verified_contacts.xlsx
+++ b/wealth_batch2_verified_contacts.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Verified Contacts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Needs Manual Research" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes &amp; Caveats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Needs Manual Research" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Verified Contacts'!$A$1:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$1:$E$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +36,11 @@
     </font>
     <font>
       <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
     </font>
   </fonts>
   <fills count="3">
@@ -63,14 +69,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,14 +447,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,358 +480,358 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Parthenon Capital</t>
+          <t>8VC</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Matt Lentz</t>
+          <t>Alex Moore</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Partner, 8VC</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>mlentz@parthenoncapital.com</t>
+          <t>amoore@8vc.com</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Stafford Capital Partners</t>
+          <t>8VC</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Kurt Faulhaber</t>
+          <t>Jake Medwell</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Co-Founder and Partner</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>kurtfaulhaber@staffordcp.com</t>
+          <t>jake@8vc.com</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stafford Capital Partners</t>
+          <t>Austin Growth Capital</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Andrew Laing</t>
+          <t>John Minter</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Principal, Head of Timber Performance, Reporting &amp; Risk</t>
+          <t>Founder and Managing Director</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>andrewlaing@staffordcp.com</t>
+          <t>jcm@austingrowthcapital.com</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TA Associates</t>
+          <t>Barton Creek Equity Partners, LLC</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Roy Burns</t>
+          <t>Tommy Odonnell</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Managing Director, Co-Head Financial Services, Americas</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>rburns@ta.com</t>
+          <t>tommy@bartoncreeklending.com</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TA Associates</t>
+          <t>CapStream Group</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Sarah Grado</t>
+          <t>Randy Finch</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Executive Assistant</t>
+          <t>Partner and Managing Director</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>sgrado@ta.com</t>
+          <t>rfinch@capstreamgroup.com</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>gatekeeper</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Escalate Capital</t>
+          <t>Capstone Capital Partners (Investing)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ross Cockrell</t>
+          <t>Ray Walter</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Co-Founder/Managing Director</t>
+          <t>CEO- Private Lender</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ross@escalatecapital.com</t>
+          <t>ray@capstonelending.com</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Escalate Capital</t>
+          <t>Capstone Capital Partners (Investing)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Kokila Lozano</t>
+          <t>Kayla Walter</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Business Owner</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>kokila@escalatecapital.com</t>
+          <t>kayla@capstonelending.com</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Revival Healthcare Capital</t>
+          <t>CenterGate Capital</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Rick Anderson</t>
+          <t>Jill Holup</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Chairman</t>
+          <t>Chief Financial Officer/Chief Operating Officer</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>rick@rvlhc.com</t>
+          <t>jholup@centergatecapital.com</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Revival Healthcare Capital</t>
+          <t>CenterGate Capital</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Sam Liang</t>
+          <t>Lewis Schoenwetter</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Operating Partner</t>
+          <t>Managing Partner</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>sam@rvlhc.com</t>
+          <t>lewis@centergatecapital.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CenterGate Capital</t>
+          <t>Escalate Capital</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Jill Holup</t>
+          <t>Ross Cockrell</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Chief Financial Officer/Chief Operating Officer</t>
+          <t>Co-Founder/Managing Director</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>jholup@centergatecapital.com</t>
+          <t>ross@escalatecapital.com</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CenterGate Capital</t>
+          <t>Escalate Capital</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Lewis Schoenwetter</t>
+          <t>Kokila Lozano</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Managing Partner</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>lewis@centergatecapital.com</t>
+          <t>kokila@escalatecapital.com</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Strattam Capital</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Bob Morse</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Founding Managing Partner</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>rmorse@strattam.com</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Escalate Capital</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Larry Bradshaw</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio Management and Compliance</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>larry@escalatecapital.com</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Strattam Capital</t>
+          <t>LiveOak Venture Partners</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Sean Williams</t>
+          <t>Krishna Srinivasan</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Vice President of Finance and Chief Compliance Officer</t>
+          <t>Founding Partner</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>swilliams@strattam.com</t>
+          <t>krishna@liveoak.vc</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
@@ -832,7 +843,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Krishna Srinivasan</t>
+          <t>Venu Shamapant</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -842,579 +853,579 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>krishna@liveoak.vc</t>
+          <t>venu@liveoak.vc</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>LiveOak Venture Partners</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Venu Shamapant</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Founding Partner</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>venu@liveoak.vc</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Mike Marcantonio</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>mike@liveoak.vc</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>S3 Ventures</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Eric Engineer</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>General Partner</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>eric@s3vc.com</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>LiveOak Venture Partners</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Creighton Hicks</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>creighton@liveoak.vc</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>S3 Ventures</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Charlie Plauche</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>General Partner</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>charlie@s3vc.com</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>LiveOak Venture Partners</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Julianna Giraldo</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>julianna@liveoak.vc</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Silverton Partners</t>
+          <t>Mainstay Global</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Kip McClanahan</t>
+          <t>Tony Frey</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>General Partner</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>kip@silvertonpartners.com</t>
+          <t>tfrey@mainstay.com</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Barton Creek Equity Partners, LLC</t>
+          <t>Next Coast Ventures LLC</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Tommy Odonnell</t>
+          <t>Michael Smerklo</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Co Founder &amp; Managing Director - Investor</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>tommy@bartoncreeklending.com</t>
+          <t>msmerklo@nextcoastventures.com</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CapStream Group</t>
+          <t>Next Coast Ventures LLC</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Randy Finch</t>
+          <t>Kaitlyn Debernardo</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Partner and Managing Director</t>
+          <t>Partner, COO and Head of Platform</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>rfinch@capstreamgroup.com</t>
+          <t>kdebernardo@nextcoastventures.com</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Trammell Ventures</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Nicole Huebner</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Chief Operating Officer</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>nhuebner@trammell.ventures</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Next Coast Ventures LLC</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Thomas Ball</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Co-Founder and Managing Director</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>tball@nextcoastventures.com</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Unknown Ventures</t>
+          <t>Parthenon Capital</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>James Gall</t>
+          <t>Matt Lentz</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>james@unknown.vc</t>
+          <t>mlentz@parthenoncapital.com</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Serent Capital</t>
+          <t>Peak Rock Capital</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Kevin Frick</t>
+          <t>Stjohn Dunne</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Principal | Operating Partner</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>kevin.frick@serentcapital.com</t>
+          <t>dunne@peakgrowthconsulting.com</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Serent Capital</t>
+          <t>Peak Rock Capital</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Carlye Nelson</t>
+          <t>Michael Hornsby</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Executive Assistant</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>carlye.nelson@serentcapital.com</t>
+          <t>hornsby@peakrockcapital.com</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>gatekeeper</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Peak Rock Capital</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Stjohn Dunne</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Principal | Operating Partner</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>dunne@peakgrowthconsulting.com</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Ryan Fitch</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>fitch@peakrockcapital.com</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Peak Rock Capital</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Michael Hornsby</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Principal</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>hornsby@peakrockcapital.com</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>John Scata</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Chief Compliance Officer</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>scata@peakrockcapital.com</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>SNH Capital Partners</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Matt Gilbreath</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Chief Operating Officer</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>mgilbreath@snhcap.com</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Peak Rock Capital</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Jung Choi</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Chief Financial Officer</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>choi@peakrockcapital.com</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SNH Capital Partners</t>
+          <t>Revival Healthcare Capital</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Jevin Sackett</t>
+          <t>Rick Anderson</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Founder &amp; Chief Executive Officer</t>
+          <t>Chairman</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>jsackett@snhcap.com</t>
+          <t>rick@rvlhc.com</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Capstone Capital Partners (Investing)</t>
+          <t>Revival Healthcare Capital</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Ray Walter</t>
+          <t>Sam Liang</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CEO- Private Lender</t>
+          <t>Operating Partner</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ray@capstonelending.com</t>
+          <t>sam@rvlhc.com</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Capstone Capital Partners (Investing)</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Kayla Walter</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Business Owner</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>kayla@capstonelending.com</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Revival Healthcare Capital</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Lisa Rainone</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Partner Head of Fund Administration and Compliance</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>lisa@rvlhc.com</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Mainstay Global</t>
+          <t>S3 Ventures</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Tony Frey</t>
+          <t>Eric Engineer</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>General Partner</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>tfrey@mainstay.com</t>
+          <t>eric@s3vc.com</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Austin Growth Capital</t>
+          <t>S3 Ventures</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>John Minter</t>
+          <t>Aaron Perman</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Founder and Managing Director</t>
+          <t>General Partner</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>jcm@austingrowthcapital.com</t>
+          <t>aaron@s3vc.com</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>8VC</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Alex Moore</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Partner, 8VC</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>amoore@8vc.com</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>S3 Ventures</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Joe Curry</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>joe@s3vc.com</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>8VC</t>
+          <t>SNH Capital Partners</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Jake Medwell</t>
+          <t>Matt Gilbreath</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Co-Founder and Partner</t>
+          <t>Chief Operating Officer</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>jake@8vc.com</t>
+          <t>mgilbreath@snhcap.com</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Sapphire Ventures</t>
+          <t>SNH Capital Partners</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Charlie Rexford</t>
+          <t>Jevin Sackett</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff to CEO</t>
+          <t>Founder &amp; Chief Executive Officer</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>charlie@sapphireventures.com</t>
+          <t>jsackett@snhcap.com</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>decision_maker+gatekeeper</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
@@ -1426,86 +1437,785 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Ralph Debernardo</t>
+          <t>Charlie Rexford</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Partner, Head of Capital Formation &amp; IR</t>
+          <t>Chief of Staff to CEO</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>ralph@sapphireventures.com</t>
+          <t>charlie@sapphireventures.com</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Next Coast Ventures LLC</t>
+          <t>Sapphire Ventures</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Michael Smerklo</t>
+          <t>Ralph Debernardo</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Co Founder &amp; Managing Director - Investor</t>
+          <t>Partner, Head of Capital Formation &amp; IR</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>msmerklo@nextcoastventures.com</t>
+          <t>ralph@sapphireventures.com</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>decision_maker</t>
+          <t>Verified</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Next Coast Ventures LLC</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Kaitlyn Debernardo</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Partner, COO and Head of Platform</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>kdebernardo@nextcoastventures.com</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>decision_maker</t>
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Sapphire Ventures</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Steve Abbott</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Partner Capital Markets</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>steve@sapphireventures.com</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Sapphire Ventures</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Abigail Johnson</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Partner Chief Operating Officer</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>abigail@sapphireventures.com</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Sapphire Ventures</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Krupa Vankayala</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Partner People and HR</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>krupa@sapphireventures.com</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Sapphire Ventures</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Monica Soliz</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Director Marketing</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>monica@sapphireventures.com</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Sapphire Ventures</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Tori Robertson</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Senior Director Marketing</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>tori@sapphireventures.com</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Serent Capital</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Kevin Frick</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>kevin.frick@serentcapital.com</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Mike Dodd</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>General Partner</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>mike@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Kip McClanahan</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>General Partner</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>kip@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Morgan Flager</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>morgan@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Roger Chen</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>roger@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Rob Taylor</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Operating Partner</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>rob@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Alyssa Dadoly</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>CFO and Partner</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>alyssa@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Matthew Saitta</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>matthew@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Addie Rasche</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>addie@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Silverton Partners</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Kristen Dumbeck</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>kristen@silvertonpartners.com</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Stafford Capital Partners</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Andrew Laing</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Principal, Head of Timber Performance, Reporting &amp; Risk</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>andrewlaing@staffordcp.com</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Stafford Capital Partners</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Lane French</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>lanefrench@staffordcp.com</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Stafford Capital Partners</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Ashley Marlow</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>NA Regional Lead</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>ashleymarlow@staffordcp.com</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Stafford Capital Partners</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Eric Rama</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Partner Stafford Timberland</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>ericrama@staffordcp.com</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Strattam Capital</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Bob Morse</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Founding Managing Partner</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>rmorse@strattam.com</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Strattam Capital</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Andrew Holden</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Principal</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>aholden@strattam.com</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>TA Associates</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Roy Burns</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Managing Director, Co-Head Financial Services, Americas</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>rburns@ta.com</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Trammell Ventures</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Nicole Huebner</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Chief Operating Officer</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>nhuebner@trammell.ventures</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Unknown Ventures</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>James Gall</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>james@unknown.vc</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E39"/>
+  <autoFilter ref="A1:E62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Peak Rock Capital</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Stjohn Dunne's email is on peakgrowthconsulting.com, not the fund's main peakrockcapital.com domain - likely an Operating Partner tied to a portfolio company. Verify before use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Capstone Capital Partners (Investing)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Apollo only has an org literally named 'Capstone Capital Partners' (capstonelending.com, a private lending shop). You added '(Investing)' to disambiguate from another entity - confirm this is actually the fund you meant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CenterGate Capital / 8VC</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Domain is confirmed but individual employees use inconsistent email formats (both first@ and flast@ seen) - no additional contacts predicted beyond the 2 directly verified, to avoid guessing wrong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>All 'Predicted (unverified)' rows</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Email built by applying the company's confirmed format to a full name sourced from the company's public team/website page, cross-validated against Apollo's obfuscated record. Not confirmed deliverable by Apollo - reasonably high confidence but not a guarantee.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1531,144 +2241,144 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>1st Commercial Credit</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Trilantic North America</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Presario Ventures</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Cotton Creek Capital</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Quake Capital Partners</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>DynEvolve Capital</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Spindletop Capital</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Keyes Capital Group</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Mako Strategies</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Altamont Capital Partners</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Sunny River Management</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Swank Investments, Inc.</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>No confident match in Apollo - find domain manually, then can re-run if needed</t>
         </is>

</xml_diff>